<commit_message>
Update model outputs 2026-08-22 08:51:26
</commit_message>
<xml_diff>
--- a/files/NRLW_futures_sim.xlsx
+++ b/files/NRLW_futures_sim.xlsx
@@ -573,16 +573,16 @@
         <v>8.7</v>
       </c>
       <c r="F2" t="n">
-        <v>96.9</v>
+        <v>97</v>
       </c>
       <c r="G2" t="n">
         <v>1.03</v>
       </c>
       <c r="H2" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="I2" t="n">
-        <v>32.36</v>
+        <v>32.95</v>
       </c>
       <c r="J2" t="n">
         <v>100</v>
@@ -595,22 +595,22 @@
       </c>
       <c r="M2"/>
       <c r="N2" t="n">
-        <v>26.3</v>
+        <v>26.7</v>
       </c>
       <c r="O2" t="n">
-        <v>3.8</v>
+        <v>3.74</v>
       </c>
       <c r="P2" t="n">
-        <v>56.6</v>
+        <v>56.8</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.77</v>
+        <v>1.76</v>
       </c>
       <c r="R2" t="n">
-        <v>32.4</v>
+        <v>32.6</v>
       </c>
       <c r="S2" t="n">
-        <v>3.09</v>
+        <v>3.06</v>
       </c>
       <c r="T2"/>
     </row>
@@ -653,13 +653,13 @@
       </c>
       <c r="M3"/>
       <c r="N3" t="n">
-        <v>70.1</v>
+        <v>69.8</v>
       </c>
       <c r="O3" t="n">
         <v>1.43</v>
       </c>
       <c r="P3" t="n">
-        <v>55.1</v>
+        <v>55.3</v>
       </c>
       <c r="Q3" t="n">
         <v>1.81</v>
@@ -668,7 +668,7 @@
         <v>26.4</v>
       </c>
       <c r="S3" t="n">
-        <v>3.79</v>
+        <v>3.78</v>
       </c>
       <c r="T3"/>
     </row>
@@ -689,16 +689,16 @@
         <v>6.8</v>
       </c>
       <c r="F4" t="n">
-        <v>58</v>
+        <v>58.4</v>
       </c>
       <c r="G4" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
       <c r="H4" t="n">
-        <v>42</v>
+        <v>41.6</v>
       </c>
       <c r="I4" t="n">
-        <v>2.38</v>
+        <v>2.4</v>
       </c>
       <c r="J4" t="n">
         <v>99.8</v>
@@ -710,25 +710,25 @@
         <v>0.2</v>
       </c>
       <c r="M4" t="n">
-        <v>555.56</v>
+        <v>588.24</v>
       </c>
       <c r="N4" t="n">
         <v>0.5</v>
       </c>
       <c r="O4" t="n">
-        <v>219.78</v>
+        <v>217.39</v>
       </c>
       <c r="P4" t="n">
-        <v>29.6</v>
+        <v>29.8</v>
       </c>
       <c r="Q4" t="n">
-        <v>3.38</v>
+        <v>3.36</v>
       </c>
       <c r="R4" t="n">
-        <v>16.3</v>
+        <v>16.4</v>
       </c>
       <c r="S4" t="n">
-        <v>6.12</v>
+        <v>6.1</v>
       </c>
       <c r="T4"/>
     </row>
@@ -749,16 +749,16 @@
         <v>7</v>
       </c>
       <c r="F5" t="n">
-        <v>66</v>
+        <v>66.2</v>
       </c>
       <c r="G5" t="n">
-        <v>1.52</v>
+        <v>1.51</v>
       </c>
       <c r="H5" t="n">
-        <v>34</v>
+        <v>33.8</v>
       </c>
       <c r="I5" t="n">
-        <v>2.94</v>
+        <v>2.96</v>
       </c>
       <c r="J5" t="n">
         <v>100</v>
@@ -777,16 +777,16 @@
         <v>50</v>
       </c>
       <c r="P5" t="n">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="Q5" t="n">
-        <v>4.36</v>
+        <v>4.35</v>
       </c>
       <c r="R5" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="S5" t="n">
-        <v>9.76</v>
+        <v>9.73</v>
       </c>
       <c r="T5"/>
     </row>
@@ -807,16 +807,16 @@
         <v>7.3</v>
       </c>
       <c r="F6" t="n">
-        <v>60.5</v>
+        <v>60</v>
       </c>
       <c r="G6" t="n">
-        <v>1.65</v>
+        <v>1.67</v>
       </c>
       <c r="H6" t="n">
-        <v>39.5</v>
+        <v>40</v>
       </c>
       <c r="I6" t="n">
-        <v>2.53</v>
+        <v>2.5</v>
       </c>
       <c r="J6" t="n">
         <v>99.8</v>
@@ -828,25 +828,25 @@
         <v>0.2</v>
       </c>
       <c r="M6" t="n">
-        <v>500</v>
+        <v>476.19</v>
       </c>
       <c r="N6" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>93.9</v>
+        <v>96.15</v>
       </c>
       <c r="P6" t="n">
-        <v>20.7</v>
+        <v>20.2</v>
       </c>
       <c r="Q6" t="n">
-        <v>4.84</v>
+        <v>4.94</v>
       </c>
       <c r="R6" t="n">
-        <v>9.2</v>
+        <v>8.9</v>
       </c>
       <c r="S6" t="n">
-        <v>10.92</v>
+        <v>11.23</v>
       </c>
       <c r="T6"/>
     </row>
@@ -867,28 +867,28 @@
         <v>5.5</v>
       </c>
       <c r="F7" t="n">
-        <v>12.9</v>
+        <v>12.4</v>
       </c>
       <c r="G7" t="n">
-        <v>7.75</v>
+        <v>8.06</v>
       </c>
       <c r="H7" t="n">
-        <v>87.1</v>
+        <v>87.6</v>
       </c>
       <c r="I7" t="n">
-        <v>1.15</v>
+        <v>1.14</v>
       </c>
       <c r="J7" t="n">
-        <v>97.1</v>
+        <v>96.9</v>
       </c>
       <c r="K7" t="n">
         <v>1.03</v>
       </c>
       <c r="L7" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="M7" t="n">
-        <v>34.84</v>
+        <v>32.52</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -897,16 +897,16 @@
         <v>4000</v>
       </c>
       <c r="P7" t="n">
-        <v>7.7</v>
+        <v>7.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>12.99</v>
+        <v>13.87</v>
       </c>
       <c r="R7" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="S7" t="n">
-        <v>35.46</v>
+        <v>38.83</v>
       </c>
       <c r="T7"/>
     </row>
@@ -927,44 +927,44 @@
         <v>5</v>
       </c>
       <c r="F8" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="G8" t="n">
-        <v>42.37</v>
+        <v>39.92</v>
       </c>
       <c r="H8" t="n">
-        <v>97.6</v>
+        <v>97.5</v>
       </c>
       <c r="I8" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
       <c r="J8" t="n">
-        <v>81.4</v>
+        <v>81.9</v>
       </c>
       <c r="K8" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
       <c r="L8" t="n">
-        <v>18.6</v>
+        <v>18.1</v>
       </c>
       <c r="M8" t="n">
-        <v>5.39</v>
+        <v>5.53</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
       </c>
       <c r="O8"/>
       <c r="P8" t="n">
-        <v>3.5</v>
+        <v>3.7</v>
       </c>
       <c r="Q8" t="n">
-        <v>28.29</v>
+        <v>26.88</v>
       </c>
       <c r="R8" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="S8" t="n">
-        <v>74.91</v>
+        <v>69.93</v>
       </c>
       <c r="T8"/>
     </row>
@@ -988,7 +988,7 @@
         <v>3.6</v>
       </c>
       <c r="G9" t="n">
-        <v>28.09</v>
+        <v>27.4</v>
       </c>
       <c r="H9" t="n">
         <v>96.4</v>
@@ -997,32 +997,32 @@
         <v>1.04</v>
       </c>
       <c r="J9" t="n">
-        <v>82.6</v>
+        <v>82.5</v>
       </c>
       <c r="K9" t="n">
         <v>1.21</v>
       </c>
       <c r="L9" t="n">
-        <v>17.4</v>
+        <v>17.5</v>
       </c>
       <c r="M9" t="n">
-        <v>5.75</v>
+        <v>5.7</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9"/>
       <c r="P9" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="Q9" t="n">
-        <v>26.77</v>
+        <v>26.6</v>
       </c>
       <c r="R9" t="n">
         <v>1.3</v>
       </c>
       <c r="S9" t="n">
-        <v>74.91</v>
+        <v>76.05</v>
       </c>
       <c r="T9"/>
     </row>
@@ -1053,13 +1053,13 @@
         <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>21</v>
+        <v>21.5</v>
       </c>
       <c r="K10" t="n">
-        <v>4.76</v>
+        <v>4.66</v>
       </c>
       <c r="L10" t="n">
-        <v>79</v>
+        <v>78.5</v>
       </c>
       <c r="M10" t="n">
         <v>1.27</v>
@@ -1072,7 +1072,7 @@
         <v>0.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>952.38</v>
+        <v>800</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -1109,13 +1109,13 @@
         <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>9.2</v>
+        <v>9.1</v>
       </c>
       <c r="K11" t="n">
-        <v>10.86</v>
+        <v>11</v>
       </c>
       <c r="L11" t="n">
-        <v>90.8</v>
+        <v>90.9</v>
       </c>
       <c r="M11" t="n">
         <v>1.1</v>
@@ -1128,7 +1128,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>2857.14</v>
+        <v>2500</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1165,16 +1165,16 @@
         <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
       <c r="K12" t="n">
-        <v>27.66</v>
+        <v>29.99</v>
       </c>
       <c r="L12" t="n">
-        <v>96.4</v>
+        <v>96.7</v>
       </c>
       <c r="M12" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -1208,7 +1208,7 @@
         <v>2.4</v>
       </c>
       <c r="E13" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -1221,16 +1221,16 @@
         <v>1</v>
       </c>
       <c r="J13" t="n">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
       <c r="K13" t="n">
-        <v>18.67</v>
+        <v>19.29</v>
       </c>
       <c r="L13" t="n">
-        <v>94.6</v>
+        <v>94.8</v>
       </c>
       <c r="M13" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update model outputs 2026-09-10 08:00:03
</commit_message>
<xml_diff>
--- a/files/NRLW_futures_sim.xlsx
+++ b/files/NRLW_futures_sim.xlsx
@@ -567,10 +567,10 @@
         <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="E2" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
@@ -593,22 +593,22 @@
       </c>
       <c r="M2"/>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O2" t="n">
-        <v>2222.22</v>
+        <v>1818.18</v>
       </c>
       <c r="P2" t="n">
-        <v>50.7</v>
+        <v>48.9</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.97</v>
+        <v>2.04</v>
       </c>
       <c r="R2" t="n">
-        <v>30.6</v>
+        <v>29.5</v>
       </c>
       <c r="S2" t="n">
-        <v>3.27</v>
+        <v>3.39</v>
       </c>
       <c r="T2"/>
     </row>
@@ -623,10 +623,10 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="E3" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -653,16 +653,16 @@
       </c>
       <c r="O3"/>
       <c r="P3" t="n">
-        <v>43.8</v>
+        <v>45.8</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.28</v>
+        <v>2.18</v>
       </c>
       <c r="R3" t="n">
-        <v>23.6</v>
+        <v>25.7</v>
       </c>
       <c r="S3" t="n">
-        <v>4.24</v>
+        <v>3.9</v>
       </c>
       <c r="T3"/>
     </row>
@@ -703,22 +703,22 @@
       </c>
       <c r="M4"/>
       <c r="N4" t="n">
-        <v>100</v>
+        <v>99.9</v>
       </c>
       <c r="O4" t="n">
         <v>1</v>
       </c>
       <c r="P4" t="n">
-        <v>39.6</v>
+        <v>38.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>2.52</v>
+        <v>2.61</v>
       </c>
       <c r="R4" t="n">
-        <v>17.9</v>
+        <v>16.7</v>
       </c>
       <c r="S4" t="n">
-        <v>5.57</v>
+        <v>6</v>
       </c>
       <c r="T4"/>
     </row>
@@ -733,10 +733,10 @@
         <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="E5" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -763,16 +763,16 @@
       </c>
       <c r="O5"/>
       <c r="P5" t="n">
-        <v>31.8</v>
+        <v>31.1</v>
       </c>
       <c r="Q5" t="n">
-        <v>3.15</v>
+        <v>3.21</v>
       </c>
       <c r="R5" t="n">
-        <v>12.6</v>
+        <v>11.8</v>
       </c>
       <c r="S5" t="n">
-        <v>7.94</v>
+        <v>8.51</v>
       </c>
       <c r="T5"/>
     </row>
@@ -787,10 +787,10 @@
         <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="E6" t="n">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
@@ -817,16 +817,16 @@
       </c>
       <c r="O6"/>
       <c r="P6" t="n">
-        <v>18.5</v>
+        <v>20</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.4</v>
+        <v>5</v>
       </c>
       <c r="R6" t="n">
-        <v>8.4</v>
+        <v>9.3</v>
       </c>
       <c r="S6" t="n">
-        <v>11.88</v>
+        <v>10.7</v>
       </c>
       <c r="T6"/>
     </row>
@@ -871,16 +871,16 @@
       </c>
       <c r="O7"/>
       <c r="P7" t="n">
-        <v>15.6</v>
+        <v>15.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>6.43</v>
+        <v>6.3</v>
       </c>
       <c r="R7" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="S7" t="n">
-        <v>14.57</v>
+        <v>14.2</v>
       </c>
       <c r="T7"/>
     </row>
@@ -965,16 +965,16 @@
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>54.9</v>
+        <v>62.3</v>
       </c>
       <c r="K9" t="n">
-        <v>1.82</v>
+        <v>1.61</v>
       </c>
       <c r="L9" t="n">
-        <v>45.1</v>
+        <v>37.7</v>
       </c>
       <c r="M9" t="n">
-        <v>2.22</v>
+        <v>2.65</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
@@ -1001,10 +1001,10 @@
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="E10" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -1017,13 +1017,13 @@
         <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
       <c r="K10" t="n">
-        <v>44.94</v>
+        <v>54.05</v>
       </c>
       <c r="L10" t="n">
-        <v>97.8</v>
+        <v>98.2</v>
       </c>
       <c r="M10" t="n">
         <v>1.02</v>
@@ -1053,10 +1053,10 @@
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="E11" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -1069,16 +1069,16 @@
         <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>42.8</v>
+        <v>35.9</v>
       </c>
       <c r="K11" t="n">
-        <v>2.33</v>
+        <v>2.79</v>
       </c>
       <c r="L11" t="n">
-        <v>57.2</v>
+        <v>64.1</v>
       </c>
       <c r="M11" t="n">
-        <v>1.75</v>
+        <v>1.56</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>

</xml_diff>